<commit_message>
Refresh synthetic sample reports
Regenerated from the e2e mock data (SAMPLES_DIR=reports): now include the
estate, mail-flow, removable-media pages and the enabled-account totals,
plus the USB and access-account action pack tabs.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/reports/sample-action-pack.xlsx
+++ b/reports/sample-action-pack.xlsx
@@ -11,17 +11,27 @@
     <sheet name="Stale accounts" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="Weak-compromised pw" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="Duplicate passwords" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="No MFA" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="Stale sensors" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="Missing sensors" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="External risks" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="No MFA - people" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="No MFA - svc &amp; mailbox" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Generic accounts" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="VPN &amp; remote-app accts" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="Stale sensors" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="Missing sensors" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="External risks" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet name="USB file writes" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet name="USB drives" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet name="USB malware" sheetId="14" state="visible" r:id="rId14"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Stale accounts'!$A$1:$K$2</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Weak-compromised pw'!$A$1:$L$2</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Stale sensors'!$A$1:$I$2</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Missing sensors'!$A$1:$I$4</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'External risks'!$A$1:$I$3</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Stale accounts'!$A$1:$M$2</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Weak-compromised pw'!$A$1:$N$2</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'VPN &amp; remote-app accts'!$A$1:$J$2</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'Stale sensors'!$A$1:$I$2</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'Missing sensors'!$A$1:$I$4</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="10" hidden="1">'External risks'!$A$1:$I$2</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="11" hidden="1">'USB file writes'!$A$1:$AC$4</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="12" hidden="1">'USB drives'!$A$1:$N$3</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="13" hidden="1">'USB malware'!$A$1:$K$2</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -447,7 +457,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C14"/>
+  <dimension ref="A1:C20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -465,7 +475,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>As at 07 October 2026. Point-in-time lists from the secops dashboard's latest collection.</t>
+          <t>As at 13 October 2026. Point-in-time lists from the secops dashboard's latest collection; USB tabs cover 07 Oct - 13 Oct 2026.</t>
         </is>
       </c>
     </row>
@@ -534,7 +544,7 @@
     <row r="8">
       <c r="A8" s="3" t="inlineStr">
         <is>
-          <t>No MFA</t>
+          <t>No MFA - people</t>
         </is>
       </c>
       <c r="B8" s="3" t="n">
@@ -542,79 +552,1289 @@
       </c>
       <c r="C8" s="3" t="inlineStr">
         <is>
-          <t>Accounts with no MFA method registered. Enrol, or disable if unused.</t>
+          <t>People (and generic logons) with no MFA method registered. Enrol, or disable if unused.</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="3" t="inlineStr">
         <is>
-          <t>Stale sensors</t>
+          <t>No MFA - svc &amp; mailbox</t>
         </is>
       </c>
       <c r="B9" s="3" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C9" s="3" t="inlineStr">
         <is>
-          <t>Managed hosts whose Falcon sensor hasn't checked in. Decommissioned: remove from Falcon. Still in use: fix the sensor -- these hosts are unprotected and unassessed.</t>
+          <t>Service accounts and mailboxes flagged for no MFA. Usually they shouldn't be cloud-synced at all: move them to an OU outside the sync scope, or exclude them from the MFA policy deliberately.</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="3" t="inlineStr">
         <is>
-          <t>Missing sensors</t>
+          <t>Generic accounts</t>
         </is>
       </c>
       <c r="B10" s="3" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="C10" s="3" t="inlineStr">
         <is>
-          <t>Machines with no Falcon sensor. Named servers/workstations are AD accounts in active use -- install a sensor or record why not. Network-only devices: identify by IP (PC, VM, or printer/IoT that can't take one).</t>
+          <t>Shared logons nobody is accountable for (from the generic-accounts groups/OUs). Replace with named accounts or disable -- enabled ones first.</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="3" t="inlineStr">
         <is>
-          <t>External risks</t>
+          <t>VPN &amp; remote-app accts</t>
         </is>
       </c>
       <c r="B11" s="3" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C11" s="3" t="inlineStr">
         <is>
-          <t>Internet-facing risks found by Hadrian: confirmed ones plus anything critical/high. Infostealer infections name the compromised accounts -- reset them and check the device.</t>
+          <t>Second accounts in the shared domain that exist only for VPN or remote apps (MANAD). Enabled + stale ones are listed first: disable them now. Legacy = in neither a VPN nor a remote-app group; confirm and remove.</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="3" t="n"/>
-      <c r="B12" s="3" t="n"/>
-      <c r="C12" s="3" t="n"/>
+      <c r="A12" s="3" t="inlineStr">
+        <is>
+          <t>Stale sensors</t>
+        </is>
+      </c>
+      <c r="B12" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="C12" s="3" t="inlineStr">
+        <is>
+          <t>Managed hosts whose Falcon sensor hasn't checked in. Decommissioned: remove from Falcon. Still in use: fix the sensor -- these hosts are unprotected and unassessed.</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="3" t="inlineStr">
         <is>
-          <t>Endpoint vulnerability lists (top remediations, worst endpoints/servers) will be added once Falcon vulnerability assessment covers the whole estate.</t>
-        </is>
-      </c>
-      <c r="B13" s="3" t="n"/>
-      <c r="C13" s="3" t="n"/>
+          <t>Missing sensors</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="C13" s="3" t="inlineStr">
+        <is>
+          <t>Machines with no Falcon sensor. Named servers/workstations are AD accounts in active use -- install a sensor or record why not. Network-only devices: identify by IP (PC, VM, or printer/IoT that can't take one).</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="3" t="inlineStr">
         <is>
+          <t>External risks</t>
+        </is>
+      </c>
+      <c r="B14" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="C14" s="3" t="inlineStr">
+        <is>
+          <t>Internet-facing risks found by Hadrian: confirmed ones plus anything critical/high. Infostealer leaks are only listed when they name one of our accounts that's still enabled -- reset it and find the device.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="3" t="inlineStr">
+        <is>
+          <t>USB file writes</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="C15" s="3" t="inlineStr">
+        <is>
+          <t>Files written to USB drives, one row per person, PC and drive, business data first. Check the flagged rows with the person or their manager: was it needed, and is the drive approved and encrypted? Email, medical images and spreadsheets/databases are the likeliest to hold patient or staff data.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="3" t="inlineStr">
+        <is>
+          <t>USB drives</t>
+        </is>
+      </c>
+      <c r="B16" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="C16" s="3" t="inlineStr">
+        <is>
+          <t>Every removable drive written to this month. Use it to decide which drives to approve (and require encryption on) and which to block in the Falcon device control policy -- shared drives first.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="3" t="inlineStr">
+        <is>
+          <t>USB malware</t>
+        </is>
+      </c>
+      <c r="B17" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="C17" s="3" t="inlineStr">
+        <is>
+          <t>Malware or unwanted software found by the scan Falcon runs when a drive is plugged in. Not quarantined: remove it and scan the drive. Repeat finds on one PC or person: find the drive and its owner.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="3" t="n"/>
+      <c r="B18" s="3" t="n"/>
+      <c r="C18" s="3" t="n"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="3" t="inlineStr">
+        <is>
+          <t>Endpoint vulnerability lists (top remediations, worst endpoints/servers) will be added once Falcon vulnerability assessment covers the whole estate.</t>
+        </is>
+      </c>
+      <c r="B19" s="3" t="n"/>
+      <c r="C19" s="3" t="n"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="3" t="inlineStr">
+        <is>
           <t>This workbook contains real account names and compromised-credential details. Keep it within the site's security contacts.</t>
         </is>
       </c>
-      <c r="B14" s="3" t="n"/>
-      <c r="C14" s="3" t="n"/>
+      <c r="B20" s="3" t="n"/>
+      <c r="C20" s="3" t="n"/>
     </row>
   </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:I4"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="18" customWidth="1" min="1" max="1"/>
+    <col width="32" customWidth="1" min="2" max="2"/>
+    <col width="15" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="16" customWidth="1" min="8" max="8"/>
+    <col width="62" customWidth="1" min="9" max="9"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="2" t="inlineStr">
+        <is>
+          <t>Site</t>
+        </is>
+      </c>
+      <c r="B1" s="2" t="inlineStr">
+        <is>
+          <t>Class</t>
+        </is>
+      </c>
+      <c r="C1" s="2" t="inlineStr">
+        <is>
+          <t>Hostname</t>
+        </is>
+      </c>
+      <c r="D1" s="2" t="inlineStr">
+        <is>
+          <t>OS</t>
+        </is>
+      </c>
+      <c r="E1" s="2" t="inlineStr">
+        <is>
+          <t>IPs</t>
+        </is>
+      </c>
+      <c r="F1" s="2" t="inlineStr">
+        <is>
+          <t>MAC vendor</t>
+        </is>
+      </c>
+      <c r="G1" s="2" t="inlineStr">
+        <is>
+          <t>Last seen</t>
+        </is>
+      </c>
+      <c r="H1" s="2" t="inlineStr">
+        <is>
+          <t>AD description</t>
+        </is>
+      </c>
+      <c r="I1" s="2" t="inlineStr">
+        <is>
+          <t>What to do</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Riverside Health</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Windows workstation, no sensor</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>RVH-WS99$</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Windows 11</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr"/>
+      <c r="G2" s="4" t="n">
+        <v>46307</v>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>Dell Latitude</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>Install a sensor; check it isn't a renamed managed host</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Lakeside Health</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>VMware NIC seen on network</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>(no hostname)</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>172.16.9.9</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>VMware, Inc.</t>
+        </is>
+      </c>
+      <c r="G3" s="4" t="n">
+        <v>46308</v>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>VM without a sensor, or an ESXi management interface: identify by IP</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Riverside Health</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Device seen on network</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>(no hostname)</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>10.1.5.5</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>Dell Inc.</t>
+        </is>
+      </c>
+      <c r="G4" s="4" t="n">
+        <v>46307</v>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>Identify by IP/MAC vendor: PC needing a sensor, or printer/IoT/appliance</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:I4"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:I2"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="18" customWidth="1" min="1" max="1"/>
+    <col width="10" customWidth="1" min="2" max="2"/>
+    <col width="21" customWidth="1" min="3" max="3"/>
+    <col width="22" customWidth="1" min="4" max="4"/>
+    <col width="45" customWidth="1" min="5" max="5"/>
+    <col width="29" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="7" customWidth="1" min="8" max="8"/>
+    <col width="13" customWidth="1" min="9" max="9"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="2" t="inlineStr">
+        <is>
+          <t>Site</t>
+        </is>
+      </c>
+      <c r="B1" s="2" t="inlineStr">
+        <is>
+          <t>Severity</t>
+        </is>
+      </c>
+      <c r="C1" s="2" t="inlineStr">
+        <is>
+          <t>Type</t>
+        </is>
+      </c>
+      <c r="D1" s="2" t="inlineStr">
+        <is>
+          <t>Category</t>
+        </is>
+      </c>
+      <c r="E1" s="2" t="inlineStr">
+        <is>
+          <t>Risk</t>
+        </is>
+      </c>
+      <c r="F1" s="2" t="inlineStr">
+        <is>
+          <t>Asset</t>
+        </is>
+      </c>
+      <c r="G1" s="2" t="inlineStr">
+        <is>
+          <t>First seen</t>
+        </is>
+      </c>
+      <c r="H1" s="2" t="inlineStr">
+        <is>
+          <t>State</t>
+        </is>
+      </c>
+      <c r="I1" s="2" t="inlineStr">
+        <is>
+          <t>Remediation</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Riverside Health</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>UnpatchedTechnology</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>unpatched-technology</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>Unpatched Apache Log4j - Actively Exploited</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>portal.riversidehealth.test</t>
+        </is>
+      </c>
+      <c r="G2" s="4" t="n">
+        <v>46303</v>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>OPEN</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>Fix it</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:I2"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:AC4"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="18" customWidth="1" min="1" max="1"/>
+    <col width="10" customWidth="1" min="2" max="2"/>
+    <col width="10" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="11" customWidth="1" min="6" max="6"/>
+    <col width="23" customWidth="1" min="7" max="7"/>
+    <col width="14" customWidth="1" min="8" max="8"/>
+    <col width="12" customWidth="1" min="9" max="9"/>
+    <col width="6" customWidth="1" min="10" max="10"/>
+    <col width="7" customWidth="1" min="11" max="11"/>
+    <col width="16" customWidth="1" min="12" max="12"/>
+    <col width="13" customWidth="1" min="13" max="13"/>
+    <col width="22" customWidth="1" min="14" max="14"/>
+    <col width="11" customWidth="1" min="15" max="15"/>
+    <col width="21" customWidth="1" min="16" max="16"/>
+    <col width="7" customWidth="1" min="17" max="17"/>
+    <col width="16" customWidth="1" min="18" max="18"/>
+    <col width="10" customWidth="1" min="19" max="19"/>
+    <col width="16" customWidth="1" min="20" max="20"/>
+    <col width="24" customWidth="1" min="21" max="21"/>
+    <col width="14" customWidth="1" min="22" max="22"/>
+    <col width="22" customWidth="1" min="23" max="23"/>
+    <col width="7" customWidth="1" min="24" max="24"/>
+    <col width="62" customWidth="1" min="25" max="25"/>
+    <col width="41" customWidth="1" min="26" max="26"/>
+    <col width="29" customWidth="1" min="27" max="27"/>
+    <col width="13" customWidth="1" min="28" max="28"/>
+    <col width="12" customWidth="1" min="29" max="29"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="2" t="inlineStr">
+        <is>
+          <t>Site</t>
+        </is>
+      </c>
+      <c r="B1" s="2" t="inlineStr">
+        <is>
+          <t>Person</t>
+        </is>
+      </c>
+      <c r="C1" s="2" t="inlineStr">
+        <is>
+          <t>Username</t>
+        </is>
+      </c>
+      <c r="D1" s="2" t="inlineStr">
+        <is>
+          <t>Title</t>
+        </is>
+      </c>
+      <c r="E1" s="2" t="inlineStr">
+        <is>
+          <t>Department</t>
+        </is>
+      </c>
+      <c r="F1" s="2" t="inlineStr">
+        <is>
+          <t>PC</t>
+        </is>
+      </c>
+      <c r="G1" s="2" t="inlineStr">
+        <is>
+          <t>USB drive</t>
+        </is>
+      </c>
+      <c r="H1" s="2" t="inlineStr">
+        <is>
+          <t>Drive serial</t>
+        </is>
+      </c>
+      <c r="I1" s="2" t="inlineStr">
+        <is>
+          <t>Connection</t>
+        </is>
+      </c>
+      <c r="J1" s="2" t="inlineStr">
+        <is>
+          <t>Days</t>
+        </is>
+      </c>
+      <c r="K1" s="2" t="inlineStr">
+        <is>
+          <t>Files</t>
+        </is>
+      </c>
+      <c r="L1" s="2" t="inlineStr">
+        <is>
+          <t>Business files</t>
+        </is>
+      </c>
+      <c r="M1" s="2" t="inlineStr">
+        <is>
+          <t>Volume (MB)</t>
+        </is>
+      </c>
+      <c r="N1" s="2" t="inlineStr">
+        <is>
+          <t>Business volume (MB)</t>
+        </is>
+      </c>
+      <c r="O1" s="2" t="inlineStr">
+        <is>
+          <t>Documents</t>
+        </is>
+      </c>
+      <c r="P1" s="2" t="inlineStr">
+        <is>
+          <t>Spreadsheets &amp; data</t>
+        </is>
+      </c>
+      <c r="Q1" s="2" t="inlineStr">
+        <is>
+          <t>Email</t>
+        </is>
+      </c>
+      <c r="R1" s="2" t="inlineStr">
+        <is>
+          <t>Medical images</t>
+        </is>
+      </c>
+      <c r="S1" s="2" t="inlineStr">
+        <is>
+          <t>Archives</t>
+        </is>
+      </c>
+      <c r="T1" s="2" t="inlineStr">
+        <is>
+          <t>Images &amp; media</t>
+        </is>
+      </c>
+      <c r="U1" s="2" t="inlineStr">
+        <is>
+          <t>Applications &amp; scripts</t>
+        </is>
+      </c>
+      <c r="V1" s="2" t="inlineStr">
+        <is>
+          <t>Design &amp; CAD</t>
+        </is>
+      </c>
+      <c r="W1" s="2" t="inlineStr">
+        <is>
+          <t>Disk images &amp; system</t>
+        </is>
+      </c>
+      <c r="X1" s="2" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="Y1" s="2" t="inlineStr">
+        <is>
+          <t>Flags</t>
+        </is>
+      </c>
+      <c r="Z1" s="2" t="inlineStr">
+        <is>
+          <t>Folders on drive</t>
+        </is>
+      </c>
+      <c r="AA1" s="2" t="inlineStr">
+        <is>
+          <t>Largest business files</t>
+        </is>
+      </c>
+      <c r="AB1" s="2" t="inlineStr">
+        <is>
+          <t>First write</t>
+        </is>
+      </c>
+      <c r="AC1" s="2" t="inlineStr">
+        <is>
+          <t>Last write</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Riverside Health</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Jo Nurse</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>jnurse</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Registered Nurse</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>Ward 3</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>RVH-WS01</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>Kingston DataTraveler</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>SER1</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>USB</t>
+        </is>
+      </c>
+      <c r="J2" t="n">
+        <v>1</v>
+      </c>
+      <c r="K2" t="n">
+        <v>4</v>
+      </c>
+      <c r="L2" t="n">
+        <v>2</v>
+      </c>
+      <c r="M2" t="n">
+        <v>2048.1</v>
+      </c>
+      <c r="N2" t="n">
+        <v>2048</v>
+      </c>
+      <c r="O2" t="n">
+        <v>0</v>
+      </c>
+      <c r="P2" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q2" t="n">
+        <v>1</v>
+      </c>
+      <c r="R2" t="n">
+        <v>0</v>
+      </c>
+      <c r="S2" t="n">
+        <v>0</v>
+      </c>
+      <c r="T2" t="n">
+        <v>2</v>
+      </c>
+      <c r="U2" t="n">
+        <v>0</v>
+      </c>
+      <c r="V2" t="n">
+        <v>0</v>
+      </c>
+      <c r="W2" t="n">
+        <v>0</v>
+      </c>
+      <c r="X2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y2" t="inlineStr">
+        <is>
+          <t>Email / mailbox data; Spreadsheets / databases; Large volume</t>
+        </is>
+      </c>
+      <c r="Z2" t="inlineStr">
+        <is>
+          <t>App\Portable, (top level), Ward\Exports</t>
+        </is>
+      </c>
+      <c r="AA2" t="inlineStr">
+        <is>
+          <t>mail.pst, Patient list.xlsx</t>
+        </is>
+      </c>
+      <c r="AB2" s="4" t="n">
+        <v>46307</v>
+      </c>
+      <c r="AC2" s="4" t="n">
+        <v>46307</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Lakeside Health</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr"/>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>LKH-SRV01</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>USB</t>
+        </is>
+      </c>
+      <c r="J3" t="n">
+        <v>1</v>
+      </c>
+      <c r="K3" t="n">
+        <v>1</v>
+      </c>
+      <c r="L3" t="n">
+        <v>1</v>
+      </c>
+      <c r="M3" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="N3" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="O3" t="n">
+        <v>0</v>
+      </c>
+      <c r="P3" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q3" t="n">
+        <v>0</v>
+      </c>
+      <c r="R3" t="n">
+        <v>0</v>
+      </c>
+      <c r="S3" t="n">
+        <v>1</v>
+      </c>
+      <c r="T3" t="n">
+        <v>0</v>
+      </c>
+      <c r="U3" t="n">
+        <v>0</v>
+      </c>
+      <c r="V3" t="n">
+        <v>0</v>
+      </c>
+      <c r="W3" t="n">
+        <v>0</v>
+      </c>
+      <c r="X3" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y3" t="inlineStr">
+        <is>
+          <t>Drive not identified; No user (system / service)</t>
+        </is>
+      </c>
+      <c r="Z3" t="inlineStr">
+        <is>
+          <t>(top level)</t>
+        </is>
+      </c>
+      <c r="AA3" t="inlineStr">
+        <is>
+          <t>backup.zip</t>
+        </is>
+      </c>
+      <c r="AB3" s="4" t="n">
+        <v>46306</v>
+      </c>
+      <c r="AC3" s="4" t="n">
+        <v>46306</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Riverside Health</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>bsmith</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>RVH-WS01</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>Kingston DataTraveler</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>SER1</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>USB</t>
+        </is>
+      </c>
+      <c r="J4" t="n">
+        <v>1</v>
+      </c>
+      <c r="K4" t="n">
+        <v>1</v>
+      </c>
+      <c r="L4" t="n">
+        <v>1</v>
+      </c>
+      <c r="M4" t="n">
+        <v>0</v>
+      </c>
+      <c r="N4" t="n">
+        <v>0</v>
+      </c>
+      <c r="O4" t="n">
+        <v>1</v>
+      </c>
+      <c r="P4" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q4" t="n">
+        <v>0</v>
+      </c>
+      <c r="R4" t="n">
+        <v>0</v>
+      </c>
+      <c r="S4" t="n">
+        <v>0</v>
+      </c>
+      <c r="T4" t="n">
+        <v>0</v>
+      </c>
+      <c r="U4" t="n">
+        <v>0</v>
+      </c>
+      <c r="V4" t="n">
+        <v>0</v>
+      </c>
+      <c r="W4" t="n">
+        <v>0</v>
+      </c>
+      <c r="X4" t="n">
+        <v>0</v>
+      </c>
+      <c r="Y4" t="inlineStr"/>
+      <c r="Z4" t="inlineStr">
+        <is>
+          <t>(top level)</t>
+        </is>
+      </c>
+      <c r="AA4" t="inlineStr">
+        <is>
+          <t>roster.docx</t>
+        </is>
+      </c>
+      <c r="AB4" s="4" t="n">
+        <v>46307</v>
+      </c>
+      <c r="AC4" s="4" t="n">
+        <v>46307</v>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:AC4"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:N3"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="18" customWidth="1" min="1" max="1"/>
+    <col width="23" customWidth="1" min="2" max="2"/>
+    <col width="8" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="8" customWidth="1" min="5" max="5"/>
+    <col width="18" customWidth="1" min="6" max="6"/>
+    <col width="5" customWidth="1" min="7" max="7"/>
+    <col width="11" customWidth="1" min="8" max="8"/>
+    <col width="7" customWidth="1" min="9" max="9"/>
+    <col width="16" customWidth="1" min="10" max="10"/>
+    <col width="13" customWidth="1" min="11" max="11"/>
+    <col width="12" customWidth="1" min="12" max="12"/>
+    <col width="12" customWidth="1" min="13" max="13"/>
+    <col width="47" customWidth="1" min="14" max="14"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="2" t="inlineStr">
+        <is>
+          <t>Site</t>
+        </is>
+      </c>
+      <c r="B1" s="2" t="inlineStr">
+        <is>
+          <t>USB drive</t>
+        </is>
+      </c>
+      <c r="C1" s="2" t="inlineStr">
+        <is>
+          <t>Serial</t>
+        </is>
+      </c>
+      <c r="D1" s="2" t="inlineStr">
+        <is>
+          <t>Connection</t>
+        </is>
+      </c>
+      <c r="E1" s="2" t="inlineStr">
+        <is>
+          <t>People</t>
+        </is>
+      </c>
+      <c r="F1" s="2" t="inlineStr">
+        <is>
+          <t>Who</t>
+        </is>
+      </c>
+      <c r="G1" s="2" t="inlineStr">
+        <is>
+          <t>PCs</t>
+        </is>
+      </c>
+      <c r="H1" s="2" t="inlineStr">
+        <is>
+          <t>Which PCs</t>
+        </is>
+      </c>
+      <c r="I1" s="2" t="inlineStr">
+        <is>
+          <t>Files</t>
+        </is>
+      </c>
+      <c r="J1" s="2" t="inlineStr">
+        <is>
+          <t>Business files</t>
+        </is>
+      </c>
+      <c r="K1" s="2" t="inlineStr">
+        <is>
+          <t>Volume (MB)</t>
+        </is>
+      </c>
+      <c r="L1" s="2" t="inlineStr">
+        <is>
+          <t>First used</t>
+        </is>
+      </c>
+      <c r="M1" s="2" t="inlineStr">
+        <is>
+          <t>Last used</t>
+        </is>
+      </c>
+      <c r="N1" s="2" t="inlineStr">
+        <is>
+          <t>Flags</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Riverside Health</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Kingston DataTraveler</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>SER1</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>USB</t>
+        </is>
+      </c>
+      <c r="E2" t="n">
+        <v>2</v>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>bsmith, Jo Nurse</t>
+        </is>
+      </c>
+      <c r="G2" t="n">
+        <v>1</v>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>RVH-WS01</t>
+        </is>
+      </c>
+      <c r="I2" t="n">
+        <v>5</v>
+      </c>
+      <c r="J2" t="n">
+        <v>3</v>
+      </c>
+      <c r="K2" t="n">
+        <v>2048.1</v>
+      </c>
+      <c r="L2" s="4" t="n">
+        <v>46307</v>
+      </c>
+      <c r="M2" s="4" t="n">
+        <v>46307</v>
+      </c>
+      <c r="N2" t="inlineStr">
+        <is>
+          <t>Shared drive</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Lakeside Health</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>USB</t>
+        </is>
+      </c>
+      <c r="E3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G3" t="n">
+        <v>1</v>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>LKH-SRV01</t>
+        </is>
+      </c>
+      <c r="I3" t="n">
+        <v>1</v>
+      </c>
+      <c r="J3" t="n">
+        <v>1</v>
+      </c>
+      <c r="K3" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="L3" s="4" t="n">
+        <v>46306</v>
+      </c>
+      <c r="M3" s="4" t="n">
+        <v>46306</v>
+      </c>
+      <c r="N3" t="inlineStr">
+        <is>
+          <t>Not identified -- one row for all such writes</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:N3"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:K2"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="18" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="10" customWidth="1" min="3" max="3"/>
+    <col width="6" customWidth="1" min="4" max="4"/>
+    <col width="27" customWidth="1" min="5" max="5"/>
+    <col width="10" customWidth="1" min="6" max="6"/>
+    <col width="11" customWidth="1" min="7" max="7"/>
+    <col width="14" customWidth="1" min="8" max="8"/>
+    <col width="13" customWidth="1" min="9" max="9"/>
+    <col width="14" customWidth="1" min="10" max="10"/>
+    <col width="11" customWidth="1" min="11" max="11"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="2" t="inlineStr">
+        <is>
+          <t>Site</t>
+        </is>
+      </c>
+      <c r="B1" s="2" t="inlineStr">
+        <is>
+          <t>Date</t>
+        </is>
+      </c>
+      <c r="C1" s="2" t="inlineStr">
+        <is>
+          <t>PC</t>
+        </is>
+      </c>
+      <c r="D1" s="2" t="inlineStr">
+        <is>
+          <t>User</t>
+        </is>
+      </c>
+      <c r="E1" s="2" t="inlineStr">
+        <is>
+          <t>Detection</t>
+        </is>
+      </c>
+      <c r="F1" s="2" t="inlineStr">
+        <is>
+          <t>Severity</t>
+        </is>
+      </c>
+      <c r="G1" s="2" t="inlineStr">
+        <is>
+          <t>File</t>
+        </is>
+      </c>
+      <c r="H1" s="2" t="inlineStr">
+        <is>
+          <t>Path</t>
+        </is>
+      </c>
+      <c r="I1" s="2" t="inlineStr">
+        <is>
+          <t>Quarantined</t>
+        </is>
+      </c>
+      <c r="J1" s="2" t="inlineStr">
+        <is>
+          <t>Alert status</t>
+        </is>
+      </c>
+      <c r="K1" s="2" t="inlineStr">
+        <is>
+          <t>Scan</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Riverside Health</t>
+        </is>
+      </c>
+      <c r="B2" s="4" t="n">
+        <v>46307</v>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>RVH-WS01</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>OnDemandScanPupAdwareHash</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>setup.exe</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>D:\setup.exe</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>new</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>completed</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:K2"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -625,20 +1845,22 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K2"/>
+  <dimension ref="A1:M2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
     <col width="14" customWidth="1" min="2" max="2"/>
     <col width="22" customWidth="1" min="3" max="3"/>
     <col width="15" customWidth="1" min="4" max="4"/>
-    <col width="11" customWidth="1" min="5" max="5"/>
-    <col width="28" customWidth="1" min="6" max="6"/>
-    <col width="9" customWidth="1" min="7" max="7"/>
-    <col width="15" customWidth="1" min="8" max="8"/>
-    <col width="23" customWidth="1" min="9" max="9"/>
-    <col width="12" customWidth="1" min="10" max="10"/>
-    <col width="20" customWidth="1" min="11" max="11"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="22" customWidth="1" min="6" max="6"/>
+    <col width="11" customWidth="1" min="7" max="7"/>
+    <col width="28" customWidth="1" min="8" max="8"/>
+    <col width="9" customWidth="1" min="9" max="9"/>
+    <col width="15" customWidth="1" min="10" max="10"/>
+    <col width="23" customWidth="1" min="11" max="11"/>
+    <col width="12" customWidth="1" min="12" max="12"/>
+    <col width="20" customWidth="1" min="13" max="13"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -664,35 +1886,45 @@
       </c>
       <c r="E1" s="2" t="inlineStr">
         <is>
+          <t>Account type</t>
+        </is>
+      </c>
+      <c r="F1" s="2" t="inlineStr">
+        <is>
+          <t>Shared-domain access</t>
+        </is>
+      </c>
+      <c r="G1" s="2" t="inlineStr">
+        <is>
           <t>Domain</t>
         </is>
       </c>
-      <c r="F1" s="2" t="inlineStr">
+      <c r="H1" s="2" t="inlineStr">
         <is>
           <t>OU</t>
         </is>
       </c>
-      <c r="G1" s="2" t="inlineStr">
+      <c r="I1" s="2" t="inlineStr">
         <is>
           <t>Enabled</t>
         </is>
       </c>
-      <c r="H1" s="2" t="inlineStr">
+      <c r="J1" s="2" t="inlineStr">
         <is>
           <t>Identity risk</t>
         </is>
       </c>
-      <c r="I1" s="2" t="inlineStr">
+      <c r="K1" s="2" t="inlineStr">
         <is>
           <t>Password last changed</t>
         </is>
       </c>
-      <c r="J1" s="2" t="inlineStr">
+      <c r="L1" s="2" t="inlineStr">
         <is>
           <t>Created</t>
         </is>
       </c>
-      <c r="K1" s="2" t="inlineStr">
+      <c r="M1" s="2" t="inlineStr">
         <is>
           <t>Other risk factors</t>
         </is>
@@ -721,38 +1953,44 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
+          <t>Service</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr"/>
+      <c r="G2" t="inlineStr">
+        <is>
           <t>RVH.LOCAL</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr">
+      <c r="H2" t="inlineStr">
         <is>
           <t>rvh.local/Service Accounts</t>
         </is>
       </c>
-      <c r="G2" t="inlineStr">
+      <c r="I2" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="H2" t="inlineStr">
+      <c r="J2" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="I2" s="4" t="n">
-        <v>45402</v>
-      </c>
-      <c r="J2" s="4" t="n">
-        <v>44302</v>
-      </c>
-      <c r="K2" t="inlineStr">
+      <c r="K2" s="4" t="n">
+        <v>45408</v>
+      </c>
+      <c r="L2" s="4" t="n">
+        <v>44308</v>
+      </c>
+      <c r="M2" t="inlineStr">
         <is>
           <t>WEAK_PASSWORD</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:K2"/>
+  <autoFilter ref="A1:M2"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -763,7 +2001,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L2"/>
+  <dimension ref="A1:N2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -771,13 +2009,15 @@
     <col width="14" customWidth="1" min="3" max="3"/>
     <col width="22" customWidth="1" min="4" max="4"/>
     <col width="15" customWidth="1" min="5" max="5"/>
-    <col width="11" customWidth="1" min="6" max="6"/>
-    <col width="28" customWidth="1" min="7" max="7"/>
-    <col width="9" customWidth="1" min="8" max="8"/>
-    <col width="15" customWidth="1" min="9" max="9"/>
-    <col width="23" customWidth="1" min="10" max="10"/>
-    <col width="12" customWidth="1" min="11" max="11"/>
-    <col width="20" customWidth="1" min="12" max="12"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="22" customWidth="1" min="7" max="7"/>
+    <col width="11" customWidth="1" min="8" max="8"/>
+    <col width="28" customWidth="1" min="9" max="9"/>
+    <col width="9" customWidth="1" min="10" max="10"/>
+    <col width="15" customWidth="1" min="11" max="11"/>
+    <col width="23" customWidth="1" min="12" max="12"/>
+    <col width="12" customWidth="1" min="13" max="13"/>
+    <col width="20" customWidth="1" min="14" max="14"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -808,35 +2048,45 @@
       </c>
       <c r="F1" s="2" t="inlineStr">
         <is>
+          <t>Account type</t>
+        </is>
+      </c>
+      <c r="G1" s="2" t="inlineStr">
+        <is>
+          <t>Shared-domain access</t>
+        </is>
+      </c>
+      <c r="H1" s="2" t="inlineStr">
+        <is>
           <t>Domain</t>
         </is>
       </c>
-      <c r="G1" s="2" t="inlineStr">
+      <c r="I1" s="2" t="inlineStr">
         <is>
           <t>OU</t>
         </is>
       </c>
-      <c r="H1" s="2" t="inlineStr">
+      <c r="J1" s="2" t="inlineStr">
         <is>
           <t>Enabled</t>
         </is>
       </c>
-      <c r="I1" s="2" t="inlineStr">
+      <c r="K1" s="2" t="inlineStr">
         <is>
           <t>Identity risk</t>
         </is>
       </c>
-      <c r="J1" s="2" t="inlineStr">
+      <c r="L1" s="2" t="inlineStr">
         <is>
           <t>Password last changed</t>
         </is>
       </c>
-      <c r="K1" s="2" t="inlineStr">
+      <c r="M1" s="2" t="inlineStr">
         <is>
           <t>Created</t>
         </is>
       </c>
-      <c r="L1" s="2" t="inlineStr">
+      <c r="N1" s="2" t="inlineStr">
         <is>
           <t>Other risk factors</t>
         </is>
@@ -870,43 +2120,337 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
+          <t>Service</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr"/>
+      <c r="H2" t="inlineStr">
+        <is>
           <t>RVH.LOCAL</t>
         </is>
       </c>
-      <c r="G2" t="inlineStr">
+      <c r="I2" t="inlineStr">
         <is>
           <t>rvh.local/Service Accounts</t>
         </is>
       </c>
-      <c r="H2" t="inlineStr">
+      <c r="J2" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="I2" t="inlineStr">
+      <c r="K2" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="J2" s="4" t="n">
-        <v>45402</v>
-      </c>
-      <c r="K2" s="4" t="n">
-        <v>44302</v>
-      </c>
-      <c r="L2" t="inlineStr">
+      <c r="L2" s="4" t="n">
+        <v>45408</v>
+      </c>
+      <c r="M2" s="4" t="n">
+        <v>44308</v>
+      </c>
+      <c r="N2" t="inlineStr">
         <is>
           <t>STALE_ACCOUNT</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:L2"/>
+  <autoFilter ref="A1:N2"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:M1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="6" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="5" customWidth="1" min="3" max="3"/>
+    <col width="15" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="22" customWidth="1" min="6" max="6"/>
+    <col width="8" customWidth="1" min="7" max="7"/>
+    <col width="4" customWidth="1" min="8" max="8"/>
+    <col width="9" customWidth="1" min="9" max="9"/>
+    <col width="15" customWidth="1" min="10" max="10"/>
+    <col width="23" customWidth="1" min="11" max="11"/>
+    <col width="9" customWidth="1" min="12" max="12"/>
+    <col width="20" customWidth="1" min="13" max="13"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="2" t="inlineStr">
+        <is>
+          <t>Site</t>
+        </is>
+      </c>
+      <c r="B1" s="2" t="inlineStr">
+        <is>
+          <t>Display name</t>
+        </is>
+      </c>
+      <c r="C1" s="2" t="inlineStr">
+        <is>
+          <t>UPN</t>
+        </is>
+      </c>
+      <c r="D1" s="2" t="inlineStr">
+        <is>
+          <t>Account (SAM)</t>
+        </is>
+      </c>
+      <c r="E1" s="2" t="inlineStr">
+        <is>
+          <t>Account type</t>
+        </is>
+      </c>
+      <c r="F1" s="2" t="inlineStr">
+        <is>
+          <t>Shared-domain access</t>
+        </is>
+      </c>
+      <c r="G1" s="2" t="inlineStr">
+        <is>
+          <t>Domain</t>
+        </is>
+      </c>
+      <c r="H1" s="2" t="inlineStr">
+        <is>
+          <t>OU</t>
+        </is>
+      </c>
+      <c r="I1" s="2" t="inlineStr">
+        <is>
+          <t>Enabled</t>
+        </is>
+      </c>
+      <c r="J1" s="2" t="inlineStr">
+        <is>
+          <t>Identity risk</t>
+        </is>
+      </c>
+      <c r="K1" s="2" t="inlineStr">
+        <is>
+          <t>Password last changed</t>
+        </is>
+      </c>
+      <c r="L1" s="2" t="inlineStr">
+        <is>
+          <t>Created</t>
+        </is>
+      </c>
+      <c r="M1" s="2" t="inlineStr">
+        <is>
+          <t>Other risk factors</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:M1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="6" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="5" customWidth="1" min="3" max="3"/>
+    <col width="15" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="22" customWidth="1" min="6" max="6"/>
+    <col width="8" customWidth="1" min="7" max="7"/>
+    <col width="4" customWidth="1" min="8" max="8"/>
+    <col width="9" customWidth="1" min="9" max="9"/>
+    <col width="15" customWidth="1" min="10" max="10"/>
+    <col width="23" customWidth="1" min="11" max="11"/>
+    <col width="9" customWidth="1" min="12" max="12"/>
+    <col width="20" customWidth="1" min="13" max="13"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="2" t="inlineStr">
+        <is>
+          <t>Site</t>
+        </is>
+      </c>
+      <c r="B1" s="2" t="inlineStr">
+        <is>
+          <t>Display name</t>
+        </is>
+      </c>
+      <c r="C1" s="2" t="inlineStr">
+        <is>
+          <t>UPN</t>
+        </is>
+      </c>
+      <c r="D1" s="2" t="inlineStr">
+        <is>
+          <t>Account (SAM)</t>
+        </is>
+      </c>
+      <c r="E1" s="2" t="inlineStr">
+        <is>
+          <t>Account type</t>
+        </is>
+      </c>
+      <c r="F1" s="2" t="inlineStr">
+        <is>
+          <t>Shared-domain access</t>
+        </is>
+      </c>
+      <c r="G1" s="2" t="inlineStr">
+        <is>
+          <t>Domain</t>
+        </is>
+      </c>
+      <c r="H1" s="2" t="inlineStr">
+        <is>
+          <t>OU</t>
+        </is>
+      </c>
+      <c r="I1" s="2" t="inlineStr">
+        <is>
+          <t>Enabled</t>
+        </is>
+      </c>
+      <c r="J1" s="2" t="inlineStr">
+        <is>
+          <t>Identity risk</t>
+        </is>
+      </c>
+      <c r="K1" s="2" t="inlineStr">
+        <is>
+          <t>Password last changed</t>
+        </is>
+      </c>
+      <c r="L1" s="2" t="inlineStr">
+        <is>
+          <t>Created</t>
+        </is>
+      </c>
+      <c r="M1" s="2" t="inlineStr">
+        <is>
+          <t>Other risk factors</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:M1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="6" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="5" customWidth="1" min="3" max="3"/>
+    <col width="15" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="22" customWidth="1" min="6" max="6"/>
+    <col width="8" customWidth="1" min="7" max="7"/>
+    <col width="4" customWidth="1" min="8" max="8"/>
+    <col width="9" customWidth="1" min="9" max="9"/>
+    <col width="15" customWidth="1" min="10" max="10"/>
+    <col width="23" customWidth="1" min="11" max="11"/>
+    <col width="9" customWidth="1" min="12" max="12"/>
+    <col width="20" customWidth="1" min="13" max="13"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="2" t="inlineStr">
+        <is>
+          <t>Site</t>
+        </is>
+      </c>
+      <c r="B1" s="2" t="inlineStr">
+        <is>
+          <t>Display name</t>
+        </is>
+      </c>
+      <c r="C1" s="2" t="inlineStr">
+        <is>
+          <t>UPN</t>
+        </is>
+      </c>
+      <c r="D1" s="2" t="inlineStr">
+        <is>
+          <t>Account (SAM)</t>
+        </is>
+      </c>
+      <c r="E1" s="2" t="inlineStr">
+        <is>
+          <t>Account type</t>
+        </is>
+      </c>
+      <c r="F1" s="2" t="inlineStr">
+        <is>
+          <t>Shared-domain access</t>
+        </is>
+      </c>
+      <c r="G1" s="2" t="inlineStr">
+        <is>
+          <t>Domain</t>
+        </is>
+      </c>
+      <c r="H1" s="2" t="inlineStr">
+        <is>
+          <t>OU</t>
+        </is>
+      </c>
+      <c r="I1" s="2" t="inlineStr">
+        <is>
+          <t>Enabled</t>
+        </is>
+      </c>
+      <c r="J1" s="2" t="inlineStr">
+        <is>
+          <t>Identity risk</t>
+        </is>
+      </c>
+      <c r="K1" s="2" t="inlineStr">
+        <is>
+          <t>Password last changed</t>
+        </is>
+      </c>
+      <c r="L1" s="2" t="inlineStr">
+        <is>
+          <t>Created</t>
+        </is>
+      </c>
+      <c r="M1" s="2" t="inlineStr">
+        <is>
+          <t>Other risk factors</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -919,13 +2463,13 @@
     <col width="14" customWidth="1" min="2" max="2"/>
     <col width="5" customWidth="1" min="3" max="3"/>
     <col width="15" customWidth="1" min="4" max="4"/>
-    <col width="8" customWidth="1" min="5" max="5"/>
-    <col width="4" customWidth="1" min="6" max="6"/>
-    <col width="9" customWidth="1" min="7" max="7"/>
-    <col width="15" customWidth="1" min="8" max="8"/>
-    <col width="23" customWidth="1" min="9" max="9"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="8" customWidth="1" min="6" max="6"/>
+    <col width="4" customWidth="1" min="7" max="7"/>
+    <col width="9" customWidth="1" min="8" max="8"/>
+    <col width="11" customWidth="1" min="9" max="9"/>
     <col width="9" customWidth="1" min="10" max="10"/>
-    <col width="20" customWidth="1" min="11" max="11"/>
+    <col width="14" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -951,27 +2495,27 @@
       </c>
       <c r="E1" s="2" t="inlineStr">
         <is>
+          <t>Account type</t>
+        </is>
+      </c>
+      <c r="F1" s="2" t="inlineStr">
+        <is>
           <t>Domain</t>
         </is>
       </c>
-      <c r="F1" s="2" t="inlineStr">
+      <c r="G1" s="2" t="inlineStr">
         <is>
           <t>OU</t>
         </is>
       </c>
-      <c r="G1" s="2" t="inlineStr">
+      <c r="H1" s="2" t="inlineStr">
         <is>
           <t>Enabled</t>
         </is>
       </c>
-      <c r="H1" s="2" t="inlineStr">
-        <is>
-          <t>Identity risk</t>
-        </is>
-      </c>
       <c r="I1" s="2" t="inlineStr">
         <is>
-          <t>Password last changed</t>
+          <t>AD groups</t>
         </is>
       </c>
       <c r="J1" s="2" t="inlineStr">
@@ -981,7 +2525,7 @@
       </c>
       <c r="K1" s="2" t="inlineStr">
         <is>
-          <t>Other risk factors</t>
+          <t>Risk factors</t>
         </is>
       </c>
     </row>
@@ -990,26 +2534,25 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K1"/>
+  <dimension ref="A1:J2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="6" customWidth="1" min="1" max="1"/>
+    <col width="18" customWidth="1" min="1" max="1"/>
     <col width="14" customWidth="1" min="2" max="2"/>
-    <col width="5" customWidth="1" min="3" max="3"/>
+    <col width="26" customWidth="1" min="3" max="3"/>
     <col width="15" customWidth="1" min="4" max="4"/>
-    <col width="8" customWidth="1" min="5" max="5"/>
-    <col width="4" customWidth="1" min="6" max="6"/>
-    <col width="9" customWidth="1" min="7" max="7"/>
-    <col width="15" customWidth="1" min="8" max="8"/>
+    <col width="10" customWidth="1" min="5" max="5"/>
+    <col width="9" customWidth="1" min="6" max="6"/>
+    <col width="7" customWidth="1" min="7" max="7"/>
+    <col width="24" customWidth="1" min="8" max="8"/>
     <col width="23" customWidth="1" min="9" max="9"/>
-    <col width="9" customWidth="1" min="10" max="10"/>
-    <col width="20" customWidth="1" min="11" max="11"/>
+    <col width="20" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1035,46 +2578,85 @@
       </c>
       <c r="E1" s="2" t="inlineStr">
         <is>
-          <t>Domain</t>
+          <t>Used for</t>
         </is>
       </c>
       <c r="F1" s="2" t="inlineStr">
         <is>
+          <t>Enabled</t>
+        </is>
+      </c>
+      <c r="G1" s="2" t="inlineStr">
+        <is>
+          <t>Stale</t>
+        </is>
+      </c>
+      <c r="H1" s="2" t="inlineStr">
+        <is>
           <t>OU</t>
         </is>
       </c>
-      <c r="G1" s="2" t="inlineStr">
-        <is>
-          <t>Enabled</t>
-        </is>
-      </c>
-      <c r="H1" s="2" t="inlineStr">
-        <is>
-          <t>Identity risk</t>
-        </is>
-      </c>
       <c r="I1" s="2" t="inlineStr">
         <is>
-          <t>Password last changed</t>
+          <t>Access groups</t>
         </is>
       </c>
       <c r="J1" s="2" t="inlineStr">
         <is>
-          <t>Created</t>
-        </is>
-      </c>
-      <c r="K1" s="2" t="inlineStr">
-        <is>
           <t>Other risk factors</t>
         </is>
       </c>
     </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Riverside Health</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Ann Nurse</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>ann@riversidehealth.test</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>ann.vpn</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>VPN</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr"/>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>shared.local/RVH/Users</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>SSL-VPN-Standard-User</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
+  <autoFilter ref="A1:J2"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1158,7 +2740,7 @@
         </is>
       </c>
       <c r="E2" s="4" t="n">
-        <v>46282</v>
+        <v>46288</v>
       </c>
       <c r="F2" t="n">
         <v>20</v>
@@ -1170,346 +2752,4 @@
   <autoFilter ref="A1:I2"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:I4"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="18" customWidth="1" min="1" max="1"/>
-    <col width="32" customWidth="1" min="2" max="2"/>
-    <col width="15" customWidth="1" min="3" max="3"/>
-    <col width="12" customWidth="1" min="4" max="4"/>
-    <col width="12" customWidth="1" min="5" max="5"/>
-    <col width="14" customWidth="1" min="6" max="6"/>
-    <col width="12" customWidth="1" min="7" max="7"/>
-    <col width="16" customWidth="1" min="8" max="8"/>
-    <col width="62" customWidth="1" min="9" max="9"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="2" t="inlineStr">
-        <is>
-          <t>Site</t>
-        </is>
-      </c>
-      <c r="B1" s="2" t="inlineStr">
-        <is>
-          <t>Class</t>
-        </is>
-      </c>
-      <c r="C1" s="2" t="inlineStr">
-        <is>
-          <t>Hostname</t>
-        </is>
-      </c>
-      <c r="D1" s="2" t="inlineStr">
-        <is>
-          <t>OS</t>
-        </is>
-      </c>
-      <c r="E1" s="2" t="inlineStr">
-        <is>
-          <t>IPs</t>
-        </is>
-      </c>
-      <c r="F1" s="2" t="inlineStr">
-        <is>
-          <t>MAC vendor</t>
-        </is>
-      </c>
-      <c r="G1" s="2" t="inlineStr">
-        <is>
-          <t>Last seen</t>
-        </is>
-      </c>
-      <c r="H1" s="2" t="inlineStr">
-        <is>
-          <t>AD description</t>
-        </is>
-      </c>
-      <c r="I1" s="2" t="inlineStr">
-        <is>
-          <t>What to do</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>Riverside Health</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>Windows workstation, no sensor</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>RVH-WS99$</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>Windows 11</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr"/>
-      <c r="G2" s="4" t="n">
-        <v>46301</v>
-      </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>Dell Latitude</t>
-        </is>
-      </c>
-      <c r="I2" t="inlineStr">
-        <is>
-          <t>Install a sensor; check it isn't a renamed managed host</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>Lakeside Health</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>VMware NIC seen on network</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>(no hostname)</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>172.16.9.9</t>
-        </is>
-      </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>VMware, Inc.</t>
-        </is>
-      </c>
-      <c r="G3" s="4" t="n">
-        <v>46302</v>
-      </c>
-      <c r="I3" t="inlineStr">
-        <is>
-          <t>VM without a sensor, or an ESXi management interface: identify by IP</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>Riverside Health</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>Device seen on network</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>(no hostname)</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>10.1.5.5</t>
-        </is>
-      </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>Dell Inc.</t>
-        </is>
-      </c>
-      <c r="G4" s="4" t="n">
-        <v>46301</v>
-      </c>
-      <c r="I4" t="inlineStr">
-        <is>
-          <t>Identify by IP/MAC vendor: PC needing a sensor, or printer/IoT/appliance</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <autoFilter ref="A1:I4"/>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:I3"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="18" customWidth="1" min="1" max="1"/>
-    <col width="10" customWidth="1" min="2" max="2"/>
-    <col width="21" customWidth="1" min="3" max="3"/>
-    <col width="22" customWidth="1" min="4" max="4"/>
-    <col width="62" customWidth="1" min="5" max="5"/>
-    <col width="29" customWidth="1" min="6" max="6"/>
-    <col width="12" customWidth="1" min="7" max="7"/>
-    <col width="10" customWidth="1" min="8" max="8"/>
-    <col width="13" customWidth="1" min="9" max="9"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="2" t="inlineStr">
-        <is>
-          <t>Site</t>
-        </is>
-      </c>
-      <c r="B1" s="2" t="inlineStr">
-        <is>
-          <t>Severity</t>
-        </is>
-      </c>
-      <c r="C1" s="2" t="inlineStr">
-        <is>
-          <t>Type</t>
-        </is>
-      </c>
-      <c r="D1" s="2" t="inlineStr">
-        <is>
-          <t>Category</t>
-        </is>
-      </c>
-      <c r="E1" s="2" t="inlineStr">
-        <is>
-          <t>Risk</t>
-        </is>
-      </c>
-      <c r="F1" s="2" t="inlineStr">
-        <is>
-          <t>Asset</t>
-        </is>
-      </c>
-      <c r="G1" s="2" t="inlineStr">
-        <is>
-          <t>First seen</t>
-        </is>
-      </c>
-      <c r="H1" s="2" t="inlineStr">
-        <is>
-          <t>State</t>
-        </is>
-      </c>
-      <c r="I1" s="2" t="inlineStr">
-        <is>
-          <t>Remediation</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>Riverside Health</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>Critical</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>UnpatchedTechnology</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>unpatched-technology</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>Unpatched Apache Log4j - Actively Exploited</t>
-        </is>
-      </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>portal.riversidehealth.test</t>
-        </is>
-      </c>
-      <c r="G2" s="4" t="n">
-        <v>46297</v>
-      </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>OPEN</t>
-        </is>
-      </c>
-      <c r="I2" t="inlineStr">
-        <is>
-          <t>Fix it</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>Riverside Health</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>Low</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>InfectedDevice</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>leaked-credentials</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>Infostealer Infection: someone@riversidehealth.test compromised</t>
-        </is>
-      </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>portal.riversidehealth.test</t>
-        </is>
-      </c>
-      <c r="G3" s="4" t="n">
-        <v>46290</v>
-      </c>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t>REOPENED</t>
-        </is>
-      </c>
-      <c r="I3" t="inlineStr">
-        <is>
-          <t>Fix it</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <autoFilter ref="A1:I3"/>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
 </file>
</xml_diff>